<commit_message>
Fix statement file detection to use correct active tab
Replace require("fs") with top-level import in statement file detection logic to resolve runtime errors in ESM module context after server restarts.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 50b14b59-b3db-470a-ad92-640b33599e59
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 37df0298-24db-493e-b51b-8811ff3bce9d
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/2aa19264-013a-4462-a379-583c1d05a569/50b14b59-b3db-470a-ad92-640b33599e59/tsaW6XY
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/uploads/statements/org-1.xlsx
+++ b/uploads/statements/org-1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Windows\ServiceProfiles\NetworkService\AppData\Local\Packages\oice_16_974fa576_32c1d314_d92\AC\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{ADEF16EE-A37B-D64F-83BA-3900B8CC7D4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1FAE5F05-BC08-414D-8B24-D851814FBB07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-60" yWindow="-60" windowWidth="15480" windowHeight="11640" xr2:uid="{DD0FE458-1732-419B-8B7D-F1B27F6E2931}"/>
+    <workbookView xWindow="-60" yWindow="-60" windowWidth="15480" windowHeight="11640" activeTab="2" xr2:uid="{DD0FE458-1732-419B-8B7D-F1B27F6E2931}"/>
   </bookViews>
   <sheets>
     <sheet name="ALL DATA" sheetId="2" r:id="rId1"/>
@@ -3065,7 +3065,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9344ABCD-347B-4F58-AC87-E58A97F033FC}">
-  <sheetPr filterMode="1">
+  <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:I299"/>
@@ -3109,7 +3109,7 @@
         <v>849</v>
       </c>
     </row>
-    <row r="2" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -3138,7 +3138,7 @@
         <v>44131</v>
       </c>
     </row>
-    <row r="3" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
@@ -3167,7 +3167,7 @@
         <v>44321</v>
       </c>
     </row>
-    <row r="4" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
@@ -3196,7 +3196,7 @@
         <v>45077</v>
       </c>
     </row>
-    <row r="5" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>2</v>
       </c>
@@ -3225,7 +3225,7 @@
         <v>45112</v>
       </c>
     </row>
-    <row r="6" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>2</v>
       </c>
@@ -3254,7 +3254,7 @@
         <v>45191</v>
       </c>
     </row>
-    <row r="7" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>2</v>
       </c>
@@ -3283,7 +3283,7 @@
         <v>45198</v>
       </c>
     </row>
-    <row r="8" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>2</v>
       </c>
@@ -3312,7 +3312,7 @@
         <v>45244</v>
       </c>
     </row>
-    <row r="9" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>2</v>
       </c>
@@ -3341,7 +3341,7 @@
         <v>45244</v>
       </c>
     </row>
-    <row r="10" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>2</v>
       </c>
@@ -3370,7 +3370,7 @@
         <v>45250</v>
       </c>
     </row>
-    <row r="11" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>2</v>
       </c>
@@ -3399,7 +3399,7 @@
         <v>45373</v>
       </c>
     </row>
-    <row r="12" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>2</v>
       </c>
@@ -3428,7 +3428,7 @@
         <v>45391</v>
       </c>
     </row>
-    <row r="13" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>2</v>
       </c>
@@ -3457,7 +3457,7 @@
         <v>45406</v>
       </c>
     </row>
-    <row r="14" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
         <v>2</v>
       </c>
@@ -3486,7 +3486,7 @@
         <v>45414</v>
       </c>
     </row>
-    <row r="15" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
         <v>2</v>
       </c>
@@ -3515,7 +3515,7 @@
         <v>45447</v>
       </c>
     </row>
-    <row r="16" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
         <v>2</v>
       </c>
@@ -3544,7 +3544,7 @@
         <v>45470</v>
       </c>
     </row>
-    <row r="17" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
         <v>2</v>
       </c>
@@ -3573,7 +3573,7 @@
         <v>45593</v>
       </c>
     </row>
-    <row r="18" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
         <v>2</v>
       </c>
@@ -3602,7 +3602,7 @@
         <v>45593</v>
       </c>
     </row>
-    <row r="19" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
         <v>2</v>
       </c>
@@ -3631,7 +3631,7 @@
         <v>45629</v>
       </c>
     </row>
-    <row r="20" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
         <v>2</v>
       </c>
@@ -3660,7 +3660,7 @@
         <v>45649</v>
       </c>
     </row>
-    <row r="21" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
         <v>2</v>
       </c>
@@ -3689,7 +3689,7 @@
         <v>45665</v>
       </c>
     </row>
-    <row r="22" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
         <v>2</v>
       </c>
@@ -3718,7 +3718,7 @@
         <v>45674</v>
       </c>
     </row>
-    <row r="23" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
         <v>2</v>
       </c>
@@ -3747,7 +3747,7 @@
         <v>45681</v>
       </c>
     </row>
-    <row r="24" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
         <v>2</v>
       </c>
@@ -3776,7 +3776,7 @@
         <v>45681</v>
       </c>
     </row>
-    <row r="25" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
         <v>2</v>
       </c>
@@ -3805,7 +3805,7 @@
         <v>45695</v>
       </c>
     </row>
-    <row r="26" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
         <v>2</v>
       </c>
@@ -3834,7 +3834,7 @@
         <v>45720</v>
       </c>
     </row>
-    <row r="27" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
         <v>2</v>
       </c>
@@ -3863,7 +3863,7 @@
         <v>45734</v>
       </c>
     </row>
-    <row r="28" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
         <v>2</v>
       </c>
@@ -3892,7 +3892,7 @@
         <v>45363</v>
       </c>
     </row>
-    <row r="29" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
         <v>2</v>
       </c>
@@ -3921,7 +3921,7 @@
         <v>45385</v>
       </c>
     </row>
-    <row r="30" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
         <v>2</v>
       </c>
@@ -3950,7 +3950,7 @@
         <v>45435</v>
       </c>
     </row>
-    <row r="31" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="s">
         <v>2</v>
       </c>
@@ -3979,7 +3979,7 @@
         <v>45440</v>
       </c>
     </row>
-    <row r="32" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
         <v>2</v>
       </c>
@@ -4008,7 +4008,7 @@
         <v>45441</v>
       </c>
     </row>
-    <row r="33" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A33" s="1" t="s">
         <v>2</v>
       </c>
@@ -4037,7 +4037,7 @@
         <v>45510</v>
       </c>
     </row>
-    <row r="34" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="s">
         <v>2</v>
       </c>
@@ -4066,7 +4066,7 @@
         <v>45526</v>
       </c>
     </row>
-    <row r="35" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="s">
         <v>2</v>
       </c>
@@ -4095,7 +4095,7 @@
         <v>45526</v>
       </c>
     </row>
-    <row r="36" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A36" s="1" t="s">
         <v>2</v>
       </c>
@@ -4124,7 +4124,7 @@
         <v>45572</v>
       </c>
     </row>
-    <row r="37" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A37" s="1" t="s">
         <v>2</v>
       </c>
@@ -4153,7 +4153,7 @@
         <v>45575</v>
       </c>
     </row>
-    <row r="38" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A38" s="1" t="s">
         <v>2</v>
       </c>
@@ -4182,7 +4182,7 @@
         <v>45583</v>
       </c>
     </row>
-    <row r="39" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A39" s="1" t="s">
         <v>2</v>
       </c>
@@ -4211,7 +4211,7 @@
         <v>45596</v>
       </c>
     </row>
-    <row r="40" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A40" s="1" t="s">
         <v>2</v>
       </c>
@@ -4240,7 +4240,7 @@
         <v>45603</v>
       </c>
     </row>
-    <row r="41" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A41" s="1" t="s">
         <v>2</v>
       </c>
@@ -4269,7 +4269,7 @@
         <v>45607</v>
       </c>
     </row>
-    <row r="42" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A42" s="1" t="s">
         <v>2</v>
       </c>
@@ -4298,7 +4298,7 @@
         <v>45649</v>
       </c>
     </row>
-    <row r="43" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A43" s="1" t="s">
         <v>2</v>
       </c>
@@ -4327,7 +4327,7 @@
         <v>45721</v>
       </c>
     </row>
-    <row r="44" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A44" s="1" t="s">
         <v>2</v>
       </c>
@@ -4356,7 +4356,7 @@
         <v>45742</v>
       </c>
     </row>
-    <row r="45" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A45" s="1" t="s">
         <v>2</v>
       </c>
@@ -4385,7 +4385,7 @@
         <v>45245</v>
       </c>
     </row>
-    <row r="46" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A46" s="1" t="s">
         <v>2</v>
       </c>
@@ -4414,7 +4414,7 @@
         <v>45254</v>
       </c>
     </row>
-    <row r="47" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A47" s="1" t="s">
         <v>2</v>
       </c>
@@ -4443,7 +4443,7 @@
         <v>45314</v>
       </c>
     </row>
-    <row r="48" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A48" s="1" t="s">
         <v>2</v>
       </c>
@@ -4472,7 +4472,7 @@
         <v>45320</v>
       </c>
     </row>
-    <row r="49" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A49" s="1" t="s">
         <v>2</v>
       </c>
@@ -4501,7 +4501,7 @@
         <v>45441</v>
       </c>
     </row>
-    <row r="50" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A50" s="1" t="s">
         <v>2</v>
       </c>
@@ -4530,7 +4530,7 @@
         <v>45453</v>
       </c>
     </row>
-    <row r="51" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A51" s="1" t="s">
         <v>2</v>
       </c>
@@ -4559,7 +4559,7 @@
         <v>45572</v>
       </c>
     </row>
-    <row r="52" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A52" s="1" t="s">
         <v>2</v>
       </c>
@@ -4588,7 +4588,7 @@
         <v>45579</v>
       </c>
     </row>
-    <row r="53" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A53" s="1" t="s">
         <v>2</v>
       </c>
@@ -4617,7 +4617,7 @@
         <v>45588</v>
       </c>
     </row>
-    <row r="54" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A54" s="1" t="s">
         <v>2</v>
       </c>
@@ -4646,7 +4646,7 @@
         <v>45604</v>
       </c>
     </row>
-    <row r="55" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A55" s="1" t="s">
         <v>2</v>
       </c>
@@ -4675,7 +4675,7 @@
         <v>45607</v>
       </c>
     </row>
-    <row r="56" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A56" s="1" t="s">
         <v>2</v>
       </c>
@@ -4704,7 +4704,7 @@
         <v>45615</v>
       </c>
     </row>
-    <row r="57" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A57" s="1" t="s">
         <v>2</v>
       </c>
@@ -4733,7 +4733,7 @@
         <v>45617</v>
       </c>
     </row>
-    <row r="58" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A58" s="1" t="s">
         <v>2</v>
       </c>
@@ -4762,7 +4762,7 @@
         <v>45622</v>
       </c>
     </row>
-    <row r="59" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A59" s="1" t="s">
         <v>2</v>
       </c>
@@ -4791,7 +4791,7 @@
         <v>45667</v>
       </c>
     </row>
-    <row r="60" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A60" s="1" t="s">
         <v>2</v>
       </c>
@@ -4820,7 +4820,7 @@
         <v>45679</v>
       </c>
     </row>
-    <row r="61" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A61" s="1" t="s">
         <v>2</v>
       </c>
@@ -4849,7 +4849,7 @@
         <v>45679</v>
       </c>
     </row>
-    <row r="62" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A62" s="1" t="s">
         <v>2</v>
       </c>
@@ -4878,7 +4878,7 @@
         <v>45684</v>
       </c>
     </row>
-    <row r="63" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A63" s="1" t="s">
         <v>2</v>
       </c>
@@ -4907,7 +4907,7 @@
         <v>45687</v>
       </c>
     </row>
-    <row r="64" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A64" s="1" t="s">
         <v>2</v>
       </c>
@@ -4936,7 +4936,7 @@
         <v>45712</v>
       </c>
     </row>
-    <row r="65" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A65" s="1" t="s">
         <v>2</v>
       </c>
@@ -4965,7 +4965,7 @@
         <v>45723</v>
       </c>
     </row>
-    <row r="66" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A66" s="1" t="s">
         <v>2</v>
       </c>
@@ -4994,7 +4994,7 @@
         <v>45733</v>
       </c>
     </row>
-    <row r="67" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A67" s="1" t="s">
         <v>2</v>
       </c>
@@ -5023,7 +5023,7 @@
         <v>45734</v>
       </c>
     </row>
-    <row r="68" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A68" s="1" t="s">
         <v>2</v>
       </c>
@@ -5052,7 +5052,7 @@
         <v>45747</v>
       </c>
     </row>
-    <row r="69" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A69" s="1" t="s">
         <v>209</v>
       </c>
@@ -5081,7 +5081,7 @@
         <v>45999</v>
       </c>
     </row>
-    <row r="70" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A70" s="1" t="s">
         <v>209</v>
       </c>
@@ -5110,7 +5110,7 @@
         <v>46014</v>
       </c>
     </row>
-    <row r="71" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A71" s="1" t="s">
         <v>209</v>
       </c>
@@ -5139,7 +5139,7 @@
         <v>44957</v>
       </c>
     </row>
-    <row r="72" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A72" s="1" t="s">
         <v>209</v>
       </c>
@@ -5168,7 +5168,7 @@
         <v>45112</v>
       </c>
     </row>
-    <row r="73" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A73" s="1" t="s">
         <v>209</v>
       </c>
@@ -5197,7 +5197,7 @@
         <v>45694</v>
       </c>
     </row>
-    <row r="74" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A74" s="1" t="s">
         <v>209</v>
       </c>
@@ -5226,7 +5226,7 @@
         <v>45901</v>
       </c>
     </row>
-    <row r="75" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A75" s="1" t="s">
         <v>209</v>
       </c>
@@ -5255,7 +5255,7 @@
         <v>45909</v>
       </c>
     </row>
-    <row r="76" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A76" s="1" t="s">
         <v>209</v>
       </c>
@@ -5284,7 +5284,7 @@
         <v>45909</v>
       </c>
     </row>
-    <row r="77" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A77" s="1" t="s">
         <v>236</v>
       </c>
@@ -5313,7 +5313,7 @@
         <v>43882</v>
       </c>
     </row>
-    <row r="78" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A78" s="1" t="s">
         <v>236</v>
       </c>
@@ -5342,7 +5342,7 @@
         <v>44501</v>
       </c>
     </row>
-    <row r="79" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A79" s="1" t="s">
         <v>236</v>
       </c>
@@ -5371,7 +5371,7 @@
         <v>44860</v>
       </c>
     </row>
-    <row r="80" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A80" s="1" t="s">
         <v>236</v>
       </c>
@@ -5400,7 +5400,7 @@
         <v>45370</v>
       </c>
     </row>
-    <row r="81" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A81" s="1" t="s">
         <v>236</v>
       </c>
@@ -5429,7 +5429,7 @@
         <v>45545</v>
       </c>
     </row>
-    <row r="82" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A82" s="1" t="s">
         <v>236</v>
       </c>
@@ -5458,7 +5458,7 @@
         <v>45672</v>
       </c>
     </row>
-    <row r="83" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A83" s="1" t="s">
         <v>236</v>
       </c>
@@ -5487,7 +5487,7 @@
         <v>45709</v>
       </c>
     </row>
-    <row r="84" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A84" s="1" t="s">
         <v>236</v>
       </c>
@@ -5516,7 +5516,7 @@
         <v>45730</v>
       </c>
     </row>
-    <row r="85" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A85" s="1" t="s">
         <v>236</v>
       </c>
@@ -7923,7 +7923,7 @@
         <v>45734</v>
       </c>
     </row>
-    <row r="168" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="168" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A168" s="1" t="s">
         <v>505</v>
       </c>
@@ -7952,7 +7952,7 @@
         <v>45483</v>
       </c>
     </row>
-    <row r="169" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="169" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A169" s="1" t="s">
         <v>505</v>
       </c>
@@ -7981,7 +7981,7 @@
         <v>45527</v>
       </c>
     </row>
-    <row r="170" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="170" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A170" s="1" t="s">
         <v>505</v>
       </c>
@@ -8010,7 +8010,7 @@
         <v>45565</v>
       </c>
     </row>
-    <row r="171" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="171" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A171" s="1" t="s">
         <v>505</v>
       </c>
@@ -8039,7 +8039,7 @@
         <v>45596</v>
       </c>
     </row>
-    <row r="172" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="172" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A172" s="1" t="s">
         <v>505</v>
       </c>
@@ -8068,7 +8068,7 @@
         <v>45741</v>
       </c>
     </row>
-    <row r="173" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="173" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A173" s="1" t="s">
         <v>505</v>
       </c>
@@ -8097,7 +8097,7 @@
         <v>45492</v>
       </c>
     </row>
-    <row r="174" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="174" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A174" s="1" t="s">
         <v>505</v>
       </c>
@@ -8126,7 +8126,7 @@
         <v>45591</v>
       </c>
     </row>
-    <row r="175" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="175" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A175" s="1" t="s">
         <v>505</v>
       </c>
@@ -8155,7 +8155,7 @@
         <v>45603</v>
       </c>
     </row>
-    <row r="176" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="176" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A176" s="1" t="s">
         <v>505</v>
       </c>
@@ -8184,7 +8184,7 @@
         <v>45631</v>
       </c>
     </row>
-    <row r="177" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="177" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A177" s="1" t="s">
         <v>505</v>
       </c>
@@ -8213,7 +8213,7 @@
         <v>45638</v>
       </c>
     </row>
-    <row r="178" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="178" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A178" s="1" t="s">
         <v>505</v>
       </c>
@@ -8242,7 +8242,7 @@
         <v>45674</v>
       </c>
     </row>
-    <row r="179" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="179" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A179" s="1" t="s">
         <v>505</v>
       </c>
@@ -8271,7 +8271,7 @@
         <v>45713</v>
       </c>
     </row>
-    <row r="180" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="180" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A180" s="1" t="s">
         <v>505</v>
       </c>
@@ -8300,7 +8300,7 @@
         <v>45737</v>
       </c>
     </row>
-    <row r="181" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="181" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A181" s="1" t="s">
         <v>505</v>
       </c>
@@ -8329,7 +8329,7 @@
         <v>45383</v>
       </c>
     </row>
-    <row r="182" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="182" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A182" s="1" t="s">
         <v>505</v>
       </c>
@@ -8358,7 +8358,7 @@
         <v>45383</v>
       </c>
     </row>
-    <row r="183" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="183" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A183" s="1" t="s">
         <v>505</v>
       </c>
@@ -8387,7 +8387,7 @@
         <v>45383</v>
       </c>
     </row>
-    <row r="184" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="184" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A184" s="1" t="s">
         <v>505</v>
       </c>
@@ -8416,7 +8416,7 @@
         <v>45383</v>
       </c>
     </row>
-    <row r="185" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="185" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A185" s="1" t="s">
         <v>505</v>
       </c>
@@ -8445,7 +8445,7 @@
         <v>45383</v>
       </c>
     </row>
-    <row r="186" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="186" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A186" s="1" t="s">
         <v>505</v>
       </c>
@@ -8474,7 +8474,7 @@
         <v>45383</v>
       </c>
     </row>
-    <row r="187" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="187" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A187" s="1" t="s">
         <v>505</v>
       </c>
@@ -8503,7 +8503,7 @@
         <v>45383</v>
       </c>
     </row>
-    <row r="188" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="188" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A188" s="1" t="s">
         <v>505</v>
       </c>
@@ -8532,7 +8532,7 @@
         <v>45383</v>
       </c>
     </row>
-    <row r="189" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="189" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A189" s="1" t="s">
         <v>505</v>
       </c>
@@ -8561,7 +8561,7 @@
         <v>45708</v>
       </c>
     </row>
-    <row r="190" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="190" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A190" s="1" t="s">
         <v>505</v>
       </c>
@@ -8590,7 +8590,7 @@
         <v>45727</v>
       </c>
     </row>
-    <row r="191" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="191" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A191" s="1" t="s">
         <v>505</v>
       </c>
@@ -8619,7 +8619,7 @@
         <v>45727</v>
       </c>
     </row>
-    <row r="192" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="192" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A192" s="1" t="s">
         <v>579</v>
       </c>
@@ -8648,7 +8648,7 @@
         <v>43454</v>
       </c>
     </row>
-    <row r="193" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="193" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A193" s="1" t="s">
         <v>579</v>
       </c>
@@ -8677,7 +8677,7 @@
         <v>43822</v>
       </c>
     </row>
-    <row r="194" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="194" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A194" s="1" t="s">
         <v>579</v>
       </c>
@@ -8706,7 +8706,7 @@
         <v>43864</v>
       </c>
     </row>
-    <row r="195" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="195" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A195" s="1" t="s">
         <v>579</v>
       </c>
@@ -8735,7 +8735,7 @@
         <v>43900</v>
       </c>
     </row>
-    <row r="196" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="196" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A196" s="1" t="s">
         <v>579</v>
       </c>
@@ -8764,7 +8764,7 @@
         <v>43906</v>
       </c>
     </row>
-    <row r="197" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="197" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A197" s="1" t="s">
         <v>579</v>
       </c>
@@ -8793,7 +8793,7 @@
         <v>44175</v>
       </c>
     </row>
-    <row r="198" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="198" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A198" s="1" t="s">
         <v>579</v>
       </c>
@@ -8822,7 +8822,7 @@
         <v>44202</v>
       </c>
     </row>
-    <row r="199" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="199" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A199" s="1" t="s">
         <v>579</v>
       </c>
@@ -8851,7 +8851,7 @@
         <v>44238</v>
       </c>
     </row>
-    <row r="200" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="200" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A200" s="1" t="s">
         <v>579</v>
       </c>
@@ -8880,7 +8880,7 @@
         <v>44301</v>
       </c>
     </row>
-    <row r="201" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="201" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A201" s="1" t="s">
         <v>579</v>
       </c>
@@ -8909,7 +8909,7 @@
         <v>44440</v>
       </c>
     </row>
-    <row r="202" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="202" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A202" s="1" t="s">
         <v>579</v>
       </c>
@@ -8938,7 +8938,7 @@
         <v>44456</v>
       </c>
     </row>
-    <row r="203" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="203" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A203" s="1" t="s">
         <v>579</v>
       </c>
@@ -8967,7 +8967,7 @@
         <v>44586</v>
       </c>
     </row>
-    <row r="204" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="204" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A204" s="1" t="s">
         <v>579</v>
       </c>
@@ -8996,7 +8996,7 @@
         <v>44601</v>
       </c>
     </row>
-    <row r="205" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="205" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A205" s="1" t="s">
         <v>579</v>
       </c>
@@ -9025,7 +9025,7 @@
         <v>44608</v>
       </c>
     </row>
-    <row r="206" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="206" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A206" s="1" t="s">
         <v>579</v>
       </c>
@@ -9054,7 +9054,7 @@
         <v>44643</v>
       </c>
     </row>
-    <row r="207" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="207" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A207" s="1" t="s">
         <v>579</v>
       </c>
@@ -9083,7 +9083,7 @@
         <v>44711</v>
       </c>
     </row>
-    <row r="208" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="208" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A208" s="1" t="s">
         <v>579</v>
       </c>
@@ -9112,7 +9112,7 @@
         <v>44868</v>
       </c>
     </row>
-    <row r="209" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="209" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A209" s="1" t="s">
         <v>579</v>
       </c>
@@ -9141,7 +9141,7 @@
         <v>44880</v>
       </c>
     </row>
-    <row r="210" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="210" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A210" s="1" t="s">
         <v>579</v>
       </c>
@@ -9170,7 +9170,7 @@
         <v>44972</v>
       </c>
     </row>
-    <row r="211" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="211" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A211" s="1" t="s">
         <v>579</v>
       </c>
@@ -9199,7 +9199,7 @@
         <v>44973</v>
       </c>
     </row>
-    <row r="212" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="212" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A212" s="1" t="s">
         <v>579</v>
       </c>
@@ -9228,7 +9228,7 @@
         <v>44981</v>
       </c>
     </row>
-    <row r="213" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="213" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A213" s="1" t="s">
         <v>579</v>
       </c>
@@ -9257,7 +9257,7 @@
         <v>44986</v>
       </c>
     </row>
-    <row r="214" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="214" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A214" s="1" t="s">
         <v>579</v>
       </c>
@@ -9286,7 +9286,7 @@
         <v>44992</v>
       </c>
     </row>
-    <row r="215" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="215" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A215" s="1" t="s">
         <v>579</v>
       </c>
@@ -9315,7 +9315,7 @@
         <v>45040</v>
       </c>
     </row>
-    <row r="216" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="216" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A216" s="1" t="s">
         <v>579</v>
       </c>
@@ -9344,7 +9344,7 @@
         <v>45043</v>
       </c>
     </row>
-    <row r="217" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="217" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A217" s="1" t="s">
         <v>579</v>
       </c>
@@ -9373,7 +9373,7 @@
         <v>45086</v>
       </c>
     </row>
-    <row r="218" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="218" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A218" s="1" t="s">
         <v>579</v>
       </c>
@@ -9402,7 +9402,7 @@
         <v>45239</v>
       </c>
     </row>
-    <row r="219" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="219" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A219" s="1" t="s">
         <v>579</v>
       </c>
@@ -9431,7 +9431,7 @@
         <v>45239</v>
       </c>
     </row>
-    <row r="220" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="220" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A220" s="1" t="s">
         <v>579</v>
       </c>
@@ -9460,7 +9460,7 @@
         <v>45239</v>
       </c>
     </row>
-    <row r="221" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="221" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A221" s="1" t="s">
         <v>579</v>
       </c>
@@ -9489,7 +9489,7 @@
         <v>45264</v>
       </c>
     </row>
-    <row r="222" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="222" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A222" s="1" t="s">
         <v>579</v>
       </c>
@@ -9518,7 +9518,7 @@
         <v>45313</v>
       </c>
     </row>
-    <row r="223" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="223" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A223" s="1" t="s">
         <v>579</v>
       </c>
@@ -9547,7 +9547,7 @@
         <v>45314</v>
       </c>
     </row>
-    <row r="224" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="224" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A224" s="1" t="s">
         <v>579</v>
       </c>
@@ -9576,7 +9576,7 @@
         <v>45341</v>
       </c>
     </row>
-    <row r="225" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="225" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A225" s="1" t="s">
         <v>579</v>
       </c>
@@ -9605,7 +9605,7 @@
         <v>45342</v>
       </c>
     </row>
-    <row r="226" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="226" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A226" s="1" t="s">
         <v>579</v>
       </c>
@@ -9634,7 +9634,7 @@
         <v>45344</v>
       </c>
     </row>
-    <row r="227" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="227" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A227" s="1" t="s">
         <v>579</v>
       </c>
@@ -9663,7 +9663,7 @@
         <v>45379</v>
       </c>
     </row>
-    <row r="228" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="228" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A228" s="1" t="s">
         <v>579</v>
       </c>
@@ -9692,7 +9692,7 @@
         <v>45404</v>
       </c>
     </row>
-    <row r="229" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="229" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A229" s="1" t="s">
         <v>579</v>
       </c>
@@ -9721,7 +9721,7 @@
         <v>45406</v>
       </c>
     </row>
-    <row r="230" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="230" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A230" s="1" t="s">
         <v>579</v>
       </c>
@@ -9750,7 +9750,7 @@
         <v>45428</v>
       </c>
     </row>
-    <row r="231" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="231" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A231" s="1" t="s">
         <v>579</v>
       </c>
@@ -9779,7 +9779,7 @@
         <v>45428</v>
       </c>
     </row>
-    <row r="232" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="232" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A232" s="1" t="s">
         <v>579</v>
       </c>
@@ -9808,7 +9808,7 @@
         <v>45428</v>
       </c>
     </row>
-    <row r="233" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="233" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A233" s="1" t="s">
         <v>579</v>
       </c>
@@ -9837,7 +9837,7 @@
         <v>45440</v>
       </c>
     </row>
-    <row r="234" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="234" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A234" s="1" t="s">
         <v>579</v>
       </c>
@@ -9866,7 +9866,7 @@
         <v>45443</v>
       </c>
     </row>
-    <row r="235" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="235" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A235" s="1" t="s">
         <v>579</v>
       </c>
@@ -9895,7 +9895,7 @@
         <v>45469</v>
       </c>
     </row>
-    <row r="236" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="236" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A236" s="1" t="s">
         <v>579</v>
       </c>
@@ -9924,7 +9924,7 @@
         <v>45470</v>
       </c>
     </row>
-    <row r="237" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="237" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A237" s="1" t="s">
         <v>579</v>
       </c>
@@ -9953,7 +9953,7 @@
         <v>45484</v>
       </c>
     </row>
-    <row r="238" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="238" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A238" s="1" t="s">
         <v>579</v>
       </c>
@@ -9982,7 +9982,7 @@
         <v>45510</v>
       </c>
     </row>
-    <row r="239" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="239" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A239" s="1" t="s">
         <v>579</v>
       </c>
@@ -10011,7 +10011,7 @@
         <v>45513</v>
       </c>
     </row>
-    <row r="240" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="240" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A240" s="1" t="s">
         <v>579</v>
       </c>
@@ -10040,7 +10040,7 @@
         <v>45517</v>
       </c>
     </row>
-    <row r="241" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="241" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A241" s="1" t="s">
         <v>579</v>
       </c>
@@ -10069,7 +10069,7 @@
         <v>45524</v>
       </c>
     </row>
-    <row r="242" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="242" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A242" s="1" t="s">
         <v>579</v>
       </c>
@@ -10098,7 +10098,7 @@
         <v>45525</v>
       </c>
     </row>
-    <row r="243" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="243" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A243" s="1" t="s">
         <v>579</v>
       </c>
@@ -10127,7 +10127,7 @@
         <v>45526</v>
       </c>
     </row>
-    <row r="244" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="244" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A244" s="1" t="s">
         <v>579</v>
       </c>
@@ -10156,7 +10156,7 @@
         <v>45552</v>
       </c>
     </row>
-    <row r="245" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="245" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A245" s="1" t="s">
         <v>579</v>
       </c>
@@ -10185,7 +10185,7 @@
         <v>45555</v>
       </c>
     </row>
-    <row r="246" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="246" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A246" s="1" t="s">
         <v>579</v>
       </c>
@@ -10214,7 +10214,7 @@
         <v>45559</v>
       </c>
     </row>
-    <row r="247" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="247" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A247" s="1" t="s">
         <v>579</v>
       </c>
@@ -10243,7 +10243,7 @@
         <v>45567</v>
       </c>
     </row>
-    <row r="248" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="248" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A248" s="1" t="s">
         <v>579</v>
       </c>
@@ -10272,7 +10272,7 @@
         <v>45569</v>
       </c>
     </row>
-    <row r="249" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="249" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A249" s="1" t="s">
         <v>579</v>
       </c>
@@ -10301,7 +10301,7 @@
         <v>45579</v>
       </c>
     </row>
-    <row r="250" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="250" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A250" s="1" t="s">
         <v>579</v>
       </c>
@@ -10330,7 +10330,7 @@
         <v>45581</v>
       </c>
     </row>
-    <row r="251" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="251" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A251" s="1" t="s">
         <v>579</v>
       </c>
@@ -10359,7 +10359,7 @@
         <v>45582</v>
       </c>
     </row>
-    <row r="252" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="252" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A252" s="1" t="s">
         <v>579</v>
       </c>
@@ -10388,7 +10388,7 @@
         <v>45587</v>
       </c>
     </row>
-    <row r="253" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="253" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A253" s="1" t="s">
         <v>579</v>
       </c>
@@ -10417,7 +10417,7 @@
         <v>45587</v>
       </c>
     </row>
-    <row r="254" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="254" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A254" s="1" t="s">
         <v>579</v>
       </c>
@@ -10446,7 +10446,7 @@
         <v>45593</v>
       </c>
     </row>
-    <row r="255" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="255" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A255" s="1" t="s">
         <v>579</v>
       </c>
@@ -10475,7 +10475,7 @@
         <v>45597</v>
       </c>
     </row>
-    <row r="256" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="256" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A256" s="1" t="s">
         <v>579</v>
       </c>
@@ -10504,7 +10504,7 @@
         <v>45600</v>
       </c>
     </row>
-    <row r="257" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="257" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A257" s="1" t="s">
         <v>579</v>
       </c>
@@ -10533,7 +10533,7 @@
         <v>45602</v>
       </c>
     </row>
-    <row r="258" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="258" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A258" s="1" t="s">
         <v>579</v>
       </c>
@@ -10562,7 +10562,7 @@
         <v>45602</v>
       </c>
     </row>
-    <row r="259" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="259" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A259" s="1" t="s">
         <v>579</v>
       </c>
@@ -10591,7 +10591,7 @@
         <v>45603</v>
       </c>
     </row>
-    <row r="260" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="260" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A260" s="1" t="s">
         <v>579</v>
       </c>
@@ -10620,7 +10620,7 @@
         <v>45615</v>
       </c>
     </row>
-    <row r="261" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="261" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A261" s="1" t="s">
         <v>579</v>
       </c>
@@ -10649,7 +10649,7 @@
         <v>45615</v>
       </c>
     </row>
-    <row r="262" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="262" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A262" s="1" t="s">
         <v>579</v>
       </c>
@@ -10678,7 +10678,7 @@
         <v>45615</v>
       </c>
     </row>
-    <row r="263" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="263" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A263" s="1" t="s">
         <v>579</v>
       </c>
@@ -10707,7 +10707,7 @@
         <v>45615</v>
       </c>
     </row>
-    <row r="264" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="264" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A264" s="1" t="s">
         <v>579</v>
       </c>
@@ -10736,7 +10736,7 @@
         <v>45628</v>
       </c>
     </row>
-    <row r="265" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="265" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A265" s="1" t="s">
         <v>579</v>
       </c>
@@ -10765,7 +10765,7 @@
         <v>45636</v>
       </c>
     </row>
-    <row r="266" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="266" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A266" s="1" t="s">
         <v>579</v>
       </c>
@@ -10794,7 +10794,7 @@
         <v>45636</v>
       </c>
     </row>
-    <row r="267" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="267" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A267" s="1" t="s">
         <v>579</v>
       </c>
@@ -10823,7 +10823,7 @@
         <v>45637</v>
       </c>
     </row>
-    <row r="268" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="268" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A268" s="1" t="s">
         <v>579</v>
       </c>
@@ -10852,7 +10852,7 @@
         <v>45673</v>
       </c>
     </row>
-    <row r="269" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="269" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A269" s="1" t="s">
         <v>579</v>
       </c>
@@ -10881,7 +10881,7 @@
         <v>45677</v>
       </c>
     </row>
-    <row r="270" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="270" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A270" s="1" t="s">
         <v>579</v>
       </c>
@@ -10910,7 +10910,7 @@
         <v>45678</v>
       </c>
     </row>
-    <row r="271" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="271" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A271" s="1" t="s">
         <v>579</v>
       </c>
@@ -10939,7 +10939,7 @@
         <v>45679</v>
       </c>
     </row>
-    <row r="272" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="272" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A272" s="1" t="s">
         <v>579</v>
       </c>
@@ -10968,7 +10968,7 @@
         <v>45695</v>
       </c>
     </row>
-    <row r="273" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="273" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A273" s="1" t="s">
         <v>579</v>
       </c>
@@ -10997,7 +10997,7 @@
         <v>45700</v>
       </c>
     </row>
-    <row r="274" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="274" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A274" s="1" t="s">
         <v>579</v>
       </c>
@@ -11026,7 +11026,7 @@
         <v>45708</v>
       </c>
     </row>
-    <row r="275" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="275" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A275" s="1" t="s">
         <v>579</v>
       </c>
@@ -11055,7 +11055,7 @@
         <v>45714</v>
       </c>
     </row>
-    <row r="276" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="276" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A276" s="1" t="s">
         <v>579</v>
       </c>
@@ -11084,7 +11084,7 @@
         <v>45733</v>
       </c>
     </row>
-    <row r="277" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="277" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A277" s="1" t="s">
         <v>579</v>
       </c>
@@ -11113,7 +11113,7 @@
         <v>45743</v>
       </c>
     </row>
-    <row r="278" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="278" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A278" s="1" t="s">
         <v>579</v>
       </c>
@@ -11142,7 +11142,7 @@
         <v>45622</v>
       </c>
     </row>
-    <row r="279" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="279" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A279" s="1" t="s">
         <v>579</v>
       </c>
@@ -11171,7 +11171,7 @@
         <v>45677</v>
       </c>
     </row>
-    <row r="280" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="280" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A280" s="1" t="s">
         <v>579</v>
       </c>
@@ -11200,7 +11200,7 @@
         <v>45680</v>
       </c>
     </row>
-    <row r="281" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="281" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A281" s="1" t="s">
         <v>790</v>
       </c>
@@ -11229,7 +11229,7 @@
         <v>45553</v>
       </c>
     </row>
-    <row r="282" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="282" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A282" s="1" t="s">
         <v>790</v>
       </c>
@@ -11258,7 +11258,7 @@
         <v>45600</v>
       </c>
     </row>
-    <row r="283" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="283" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A283" s="1" t="s">
         <v>790</v>
       </c>
@@ -11287,7 +11287,7 @@
         <v>45695</v>
       </c>
     </row>
-    <row r="284" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="284" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A284" s="1" t="s">
         <v>790</v>
       </c>
@@ -11316,7 +11316,7 @@
         <v>45055</v>
       </c>
     </row>
-    <row r="285" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="285" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A285" s="1" t="s">
         <v>790</v>
       </c>
@@ -11345,7 +11345,7 @@
         <v>45089</v>
       </c>
     </row>
-    <row r="286" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="286" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A286" s="1" t="s">
         <v>790</v>
       </c>
@@ -11374,7 +11374,7 @@
         <v>45104</v>
       </c>
     </row>
-    <row r="287" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="287" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A287" s="1" t="s">
         <v>790</v>
       </c>
@@ -11403,7 +11403,7 @@
         <v>45208</v>
       </c>
     </row>
-    <row r="288" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="288" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A288" s="1" t="s">
         <v>790</v>
       </c>
@@ -11432,7 +11432,7 @@
         <v>45223</v>
       </c>
     </row>
-    <row r="289" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="289" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A289" s="1" t="s">
         <v>790</v>
       </c>
@@ -11461,7 +11461,7 @@
         <v>45259</v>
       </c>
     </row>
-    <row r="290" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="290" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A290" s="1" t="s">
         <v>790</v>
       </c>
@@ -11490,7 +11490,7 @@
         <v>45261</v>
       </c>
     </row>
-    <row r="291" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="291" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A291" s="1" t="s">
         <v>790</v>
       </c>
@@ -11519,7 +11519,7 @@
         <v>45316</v>
       </c>
     </row>
-    <row r="292" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="292" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A292" s="1" t="s">
         <v>790</v>
       </c>
@@ -11548,7 +11548,7 @@
         <v>45316</v>
       </c>
     </row>
-    <row r="293" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="293" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A293" s="1" t="s">
         <v>790</v>
       </c>
@@ -11577,7 +11577,7 @@
         <v>45316</v>
       </c>
     </row>
-    <row r="294" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="294" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A294" s="1" t="s">
         <v>790</v>
       </c>
@@ -11606,7 +11606,7 @@
         <v>45316</v>
       </c>
     </row>
-    <row r="295" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="295" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A295" s="1" t="s">
         <v>790</v>
       </c>
@@ -11635,7 +11635,7 @@
         <v>45342</v>
       </c>
     </row>
-    <row r="296" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="296" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A296" s="1" t="s">
         <v>790</v>
       </c>
@@ -11664,7 +11664,7 @@
         <v>45462</v>
       </c>
     </row>
-    <row r="297" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="297" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A297" s="1" t="s">
         <v>790</v>
       </c>
@@ -11693,7 +11693,7 @@
         <v>45621</v>
       </c>
     </row>
-    <row r="298" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="298" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A298" s="1" t="s">
         <v>790</v>
       </c>
@@ -11722,7 +11722,7 @@
         <v>45700</v>
       </c>
     </row>
-    <row r="299" spans="1:9" hidden="1" x14ac:dyDescent="0.2">
+    <row r="299" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A299" s="6"/>
       <c r="B299" s="6"/>
       <c r="C299" s="6"/>
@@ -11737,12 +11737,7 @@
       <c r="I299" s="6"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I299" xr:uid="{15049A58-7C55-4735-9C3E-ACD0DBADD052}">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="LITI"/>
-      </filters>
-    </filterColumn>
+  <autoFilter ref="A1:I1" xr:uid="{15049A58-7C55-4735-9C3E-ACD0DBADD052}">
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I299">
       <sortCondition ref="A1"/>
     </sortState>

</xml_diff>

<commit_message>
Restrict statement uploads to Excel files only
Update server and client-side code to exclusively allow .xls and .xlsx file uploads for statements, rejecting all other file types including CSV.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 50b14b59-b3db-470a-ad92-640b33599e59
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 31e8ec07-cbf2-4921-a42d-8306ff7879aa
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/2aa19264-013a-4462-a379-583c1d05a569/50b14b59-b3db-470a-ad92-640b33599e59/tsaW6XY
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/uploads/statements/org-1.xlsx
+++ b/uploads/statements/org-1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Windows\ServiceProfiles\NetworkService\AppData\Local\Packages\oice_16_974fa576_32c1d314_d92\AC\Temp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1FAE5F05-BC08-414D-8B24-D851814FBB07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A42E7679-E208-EF44-8BD0-950D15C75457}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-60" yWindow="-60" windowWidth="15480" windowHeight="11640" activeTab="2" xr2:uid="{DD0FE458-1732-419B-8B7D-F1B27F6E2931}"/>
+    <workbookView xWindow="-60" yWindow="-60" windowWidth="15480" windowHeight="11640" activeTab="7" xr2:uid="{DD0FE458-1732-419B-8B7D-F1B27F6E2931}"/>
   </bookViews>
   <sheets>
     <sheet name="ALL DATA" sheetId="2" r:id="rId1"/>

</xml_diff>